<commit_message>
feat(schema): add in-toto digests, issuer results and VSA field rules
Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/slsa.xlsx
+++ b/project/excel/slsa.xlsx
@@ -8,39 +8,43 @@
   </bookViews>
   <sheets>
     <sheet name="InTotoDigestSet" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="InTotoAnnotation" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="InTotoResourceDescriptor" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="InTotoStatement" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="SlsaProducer" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="SlsaConsumer" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="SlsaVerifier" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="SlsaInfrastructureProvider" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="SlsaBuildPlatform" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="SlsaControlPlane" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="SlsaComponentVersion" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="SlsaPackageRegistry" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="SlsaPackage" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="SlsaBuildProvenance" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="SlsaBuildDefinition" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="SlsaBuildParameter" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="SlsaRunDetails" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="SlsaBuildMetadata" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="SlsaVerificationSummary" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="SlsaDependencyLevelCount" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="SlsaSourceControlSystem" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="SlsaSourceRepository" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="SlsaSourceRevision" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="SlsaNamedReference" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="SlsaBranch" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="SlsaTag" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="SlsaSourceProvenance" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="SlsaDependencyInventory" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="SlsaBuildImageProducer" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="SlsaBuildImage" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="SlsaMeasurement" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="SlsaBuildEnvironmentAttestation" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="SlsaAdoptionMetadata" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="SlsaDocument" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="InTotoAdditionalDigest" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="InTotoAnnotation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="InTotoResourceDescriptor" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="InTotoStatementSubject" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="InTotoStatement" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="SlsaProducer" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="SlsaConsumer" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="SlsaVerifier" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="SlsaInfrastructureProvider" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="SlsaBuildPlatform" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="SlsaControlPlane" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="SlsaComponentVersion" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="SlsaPackageRegistry" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="SlsaPackage" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="SlsaBuildProvenance" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="SlsaBuildDefinition" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="SlsaBuildParameter" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="SlsaRunDetails" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="SlsaBuildMetadata" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="SlsaVerificationSummary" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="SlsaDependencyLevelCount" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="SlsaVerificationSummaryPolicy" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="SlsaVerificationSummaryI_21b431" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="SlsaSourceControlSystem" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="SlsaSourceRepository" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="SlsaSourceRevision" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="SlsaNamedReference" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="SlsaBranch" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="SlsaTag" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="SlsaSourceProvenance" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="SlsaDependencyInventory" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="SlsaBuildImageProducer" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="SlsaBuildImage" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="SlsaMeasurement" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="SlsaBuildEnvironmentAttestation" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="SlsaAdoptionMetadata" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="SlsaDocument" sheetId="38" state="visible" r:id="rId38"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -446,42 +450,214 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:Y1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>sha256</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sha224</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>sha384</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>sha512</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>sha512_224</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>sha512_256</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>sha3_224</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>sha3_256</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>sha3_384</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>sha3_512</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>shake128</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>shake256</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>blake2b</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>blake2s</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>ripemd160</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>sm3</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>gost</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>sha1</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>md5</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>dir_hash</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>git_commit</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>git_tree</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>git_blob</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>git_tag</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>additional_digests</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>party_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>party_name</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>sha256</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>sha512</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>git_commit</t>
+          <t>component_versions</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>builder_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>build_level</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>git_tree</t>
+          <t>hosted</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>dir_hash</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+          <t>builder_dependencies</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"SLSA_BUILD_LEVEL_0,SLSA_BUILD_LEVEL_1,SLSA_BUILD_LEVEL_2,SLSA_BUILD_LEVEL_3"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -502,7 +678,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -528,7 +704,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -554,7 +730,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -600,7 +776,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -631,7 +807,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -682,7 +858,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -708,7 +884,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -739,7 +915,33 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -770,7 +972,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -846,7 +1048,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -858,21 +1060,144 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>annotation_key</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>annotation_values</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+          <t>verified_level</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>dependency_count</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>resource_uri</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>digest</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>resource_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>download_location</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>media_type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>content</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>annotations</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>resource_uri</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>digest</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>resource_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>download_location</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>media_type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>content</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>annotations</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>scs_uri</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -884,53 +1209,6 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>verified_level</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>dependency_count</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>scs_uri</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
           <t>repository_uri</t>
         </is>
       </c>
@@ -945,7 +1223,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1004,7 +1282,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1045,7 +1323,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1086,7 +1364,33 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>annotation_key</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>annotation_values</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1127,7 +1431,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1158,7 +1462,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1194,7 +1498,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1220,53 +1524,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>resource_uri</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>digest</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>resource_name</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>download_location</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>media_type</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>annotations</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1307,7 +1565,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1333,7 +1591,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1379,7 +1637,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1413,13 +1671,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L1"/>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1440,56 +1698,112 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>control_planes</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>packages</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>package_registries</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>source_control_systems</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>source_repositories</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>source_revisions</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>named_references</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>build_images</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>dependency_inventories</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>adoption_metadata</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>resource_uri</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>digest</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>resource_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>download_location</t>
+        </is>
+      </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>package_registries</t>
+          <t>media_type</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>source_control_systems</t>
+          <t>content</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>source_repositories</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>source_revisions</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>named_references</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>build_images</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>dependency_inventories</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>adoption_metadata</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+          <t>annotations</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1501,6 +1815,57 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>resource_uri</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>digest</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>resource_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>download_location</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>media_type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>content</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>annotations</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t>statement_type</t>
         </is>
       </c>
@@ -1540,7 +1905,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1571,7 +1936,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1597,7 +1962,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1631,76 +1996,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>party_type</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>party_name</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>component_versions</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>builder_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>build_level</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>hosted</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>builder_dependencies</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"SLSA_BUILD_LEVEL_0,SLSA_BUILD_LEVEL_1,SLSA_BUILD_LEVEL_2,SLSA_BUILD_LEVEL_3"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(schema): add in-toto digests, issuer results and VSA field rules (#28)
* feat(schema): add in-toto digests, issuer results and VSA field rules

Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>

* docs(lokf): refresh the bundle for the schema review

Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>

* fix: correct the README rename sentence and the spell-check lists

Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>

* docs(lokf): resolve the README rename question

Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>

* ci(lint): skip Zenodo DOIs, which time out for ci runners

Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>

---------

Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/slsa.xlsx
+++ b/project/excel/slsa.xlsx
@@ -8,39 +8,43 @@
   </bookViews>
   <sheets>
     <sheet name="InTotoDigestSet" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="InTotoAnnotation" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="InTotoResourceDescriptor" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="InTotoStatement" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="SlsaProducer" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="SlsaConsumer" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="SlsaVerifier" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="SlsaInfrastructureProvider" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="SlsaBuildPlatform" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="SlsaControlPlane" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="SlsaComponentVersion" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="SlsaPackageRegistry" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="SlsaPackage" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="SlsaBuildProvenance" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="SlsaBuildDefinition" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="SlsaBuildParameter" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="SlsaRunDetails" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="SlsaBuildMetadata" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="SlsaVerificationSummary" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="SlsaDependencyLevelCount" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="SlsaSourceControlSystem" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="SlsaSourceRepository" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="SlsaSourceRevision" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="SlsaNamedReference" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="SlsaBranch" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="SlsaTag" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="SlsaSourceProvenance" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="SlsaDependencyInventory" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="SlsaBuildImageProducer" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="SlsaBuildImage" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="SlsaMeasurement" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="SlsaBuildEnvironmentAttestation" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="SlsaAdoptionMetadata" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="SlsaDocument" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="InTotoAdditionalDigest" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="InTotoAnnotation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="InTotoResourceDescriptor" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="InTotoStatementSubject" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="InTotoStatement" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="SlsaProducer" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="SlsaConsumer" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="SlsaVerifier" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="SlsaInfrastructureProvider" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="SlsaBuildPlatform" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="SlsaControlPlane" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="SlsaComponentVersion" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="SlsaPackageRegistry" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="SlsaPackage" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="SlsaBuildProvenance" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="SlsaBuildDefinition" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="SlsaBuildParameter" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="SlsaRunDetails" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="SlsaBuildMetadata" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="SlsaVerificationSummary" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="SlsaDependencyLevelCount" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="SlsaVerificationSummaryPolicy" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="SlsaVerificationSummaryI_21b431" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="SlsaSourceControlSystem" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="SlsaSourceRepository" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="SlsaSourceRevision" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="SlsaNamedReference" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="SlsaBranch" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="SlsaTag" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="SlsaSourceProvenance" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="SlsaDependencyInventory" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="SlsaBuildImageProducer" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="SlsaBuildImage" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="SlsaMeasurement" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="SlsaBuildEnvironmentAttestation" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="SlsaAdoptionMetadata" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="SlsaDocument" sheetId="38" state="visible" r:id="rId38"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -446,42 +450,214 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:Y1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>sha256</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sha224</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>sha384</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>sha512</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>sha512_224</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>sha512_256</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>sha3_224</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>sha3_256</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>sha3_384</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>sha3_512</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>shake128</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>shake256</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>blake2b</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>blake2s</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>ripemd160</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>sm3</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>gost</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>sha1</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>md5</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>dir_hash</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>git_commit</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>git_tree</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>git_blob</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>git_tag</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>additional_digests</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>party_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>party_name</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>sha256</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>sha512</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>git_commit</t>
+          <t>component_versions</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>builder_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>build_level</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>git_tree</t>
+          <t>hosted</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>dir_hash</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+          <t>builder_dependencies</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"SLSA_BUILD_LEVEL_0,SLSA_BUILD_LEVEL_1,SLSA_BUILD_LEVEL_2,SLSA_BUILD_LEVEL_3"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -502,7 +678,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -528,7 +704,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -554,7 +730,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -600,7 +776,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -631,7 +807,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -682,7 +858,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -708,7 +884,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -739,7 +915,33 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -770,7 +972,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -846,7 +1048,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -858,21 +1060,144 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>annotation_key</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>annotation_values</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+          <t>verified_level</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>dependency_count</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>resource_uri</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>digest</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>resource_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>download_location</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>media_type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>content</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>annotations</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>resource_uri</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>digest</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>resource_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>download_location</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>media_type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>content</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>annotations</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>scs_uri</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -884,53 +1209,6 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>verified_level</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>dependency_count</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>scs_uri</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
           <t>repository_uri</t>
         </is>
       </c>
@@ -945,7 +1223,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1004,7 +1282,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1045,7 +1323,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1086,7 +1364,33 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>annotation_key</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>annotation_values</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1127,7 +1431,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1158,7 +1462,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1194,7 +1498,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1220,53 +1524,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>resource_uri</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>digest</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>resource_name</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>download_location</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>media_type</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>annotations</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1307,7 +1565,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1333,7 +1591,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1379,7 +1637,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1413,13 +1671,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L1"/>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1440,56 +1698,112 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>control_planes</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>packages</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>package_registries</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>source_control_systems</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>source_repositories</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>source_revisions</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>named_references</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>build_images</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>dependency_inventories</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>adoption_metadata</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>resource_uri</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>digest</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>resource_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>download_location</t>
+        </is>
+      </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>package_registries</t>
+          <t>media_type</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>source_control_systems</t>
+          <t>content</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>source_repositories</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>source_revisions</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>named_references</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>build_images</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>dependency_inventories</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>adoption_metadata</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+          <t>annotations</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1501,6 +1815,57 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>resource_uri</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>digest</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>resource_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>download_location</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>media_type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>content</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>annotations</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t>statement_type</t>
         </is>
       </c>
@@ -1540,7 +1905,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1571,7 +1936,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1597,7 +1962,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1631,76 +1996,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>party_type</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>party_name</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>component_versions</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>builder_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>build_level</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>hosted</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>builder_dependencies</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"SLSA_BUILD_LEVEL_0,SLSA_BUILD_LEVEL_1,SLSA_BUILD_LEVEL_2,SLSA_BUILD_LEVEL_3"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>